<commit_message>
bis-2879: Reconstruct and write collection types
</commit_message>
<xml_diff>
--- a/app-ro-crate-openbis/src/test/resources/json2excel/openbis_test_ro_out.xlsx
+++ b/app-ro-crate-openbis/src/test/resources/json2excel/openbis_test_ro_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="152">
   <si>
     <t>SAMPLE_TYPE</t>
   </si>
@@ -275,16 +275,22 @@
     <t>COLLECTION</t>
   </si>
   <si>
-    <t>General info</t>
-  </si>
-  <si>
     <t>DEFAULT_OBJECT_TYPE</t>
   </si>
   <si>
-    <t>Default object type</t>
-  </si>
-  <si>
-    <t>Enter the code of the object type for which the collection is used</t>
+    <t>openBIS:hasDEFAULT_OBJECT_TYPE</t>
+  </si>
+  <si>
+    <t>openBIS:hasDEFAULT_OBJECT_TYPE: DEFAULT_OBJECT_TYPE</t>
+  </si>
+  <si>
+    <t>DEFAULT_COLLECTION_VIEW</t>
+  </si>
+  <si>
+    <t>openBIS:hasDEFAULT_COLLECTION_VIEW</t>
+  </si>
+  <si>
+    <t>openBIS:hasDEFAULT_COLLECTION_VIEW: DEFAULT_COLLECTION_VIEW</t>
   </si>
   <si>
     <t>SPACE</t>
@@ -323,34 +329,34 @@
     <t>Project</t>
   </si>
   <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATION_COLLECTION</t>
-  </si>
-  <si>
-    <t>PUBLICATION_COLLECTION</t>
-  </si>
-  <si>
-    <t>Unknown Collection</t>
-  </si>
-  <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATION_CREATOR_COLLECTION</t>
-  </si>
-  <si>
-    <t>PUBLICATION_CREATOR_COLLECTION</t>
-  </si>
-  <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATION_PUBLISHER_COLLECTION</t>
-  </si>
-  <si>
-    <t>PUBLICATION_PUBLISHER_COLLECTION</t>
-  </si>
-  <si>
-    <t>/DEFAULT/DEFAULT/PUBLICATION_COLLECTION</t>
-  </si>
-  <si>
-    <t>/DEFAULT/DEFAULT/PUBLICATION_CREATOR_COLLECTION</t>
-  </si>
-  <si>
-    <t>/DEFAULT/DEFAULT/PUBLICATION_PUBLISHER_COLLECTION</t>
+    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATIONS_COLLECTION</t>
+  </si>
+  <si>
+    <t>PUBLICATIONS_COLLECTION</t>
+  </si>
+  <si>
+    <t>Publications Collection</t>
+  </si>
+  <si>
+    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATIONS_CREATOR_COLLECTION</t>
+  </si>
+  <si>
+    <t>PUBLICATIONS_CREATOR_COLLECTION</t>
+  </si>
+  <si>
+    <t>Publications creator collection</t>
+  </si>
+  <si>
+    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATIONS_PUBLISHER_COLLECTION</t>
+  </si>
+  <si>
+    <t>PUBLICATIONS_PUBLISHER_COLLECTION</t>
+  </si>
+  <si>
+    <t>Publications Publisher Collection</t>
+  </si>
+  <si>
+    <t>LIST_VIEW</t>
   </si>
   <si>
     <t>Sample type</t>
@@ -374,9 +380,6 @@
     <t>PUBCREA22</t>
   </si>
   <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATIONS_CREATOR_COLLECTION</t>
-  </si>
-  <si>
     <t>Elhacham</t>
   </si>
   <si>
@@ -416,9 +419,6 @@
     <t>PUBPUB24</t>
   </si>
   <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATIONS_PUBLISHER_COLLECTION</t>
-  </si>
-  <si>
     <t>https://www.nature.com</t>
   </si>
   <si>
@@ -435,9 +435,6 @@
   </si>
   <si>
     <t>PUB25</t>
-  </si>
-  <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATIONS_COLLECTION</t>
   </si>
   <si>
     <t>Global human-made mass exceeds all living biomass</t>
@@ -1317,7 +1314,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1378,10 +1375,31 @@
       <c r="J4" t="s" s="1">
         <v>19</v>
       </c>
+      <c r="K4" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="L4" t="s" s="1">
+        <v>7</v>
+      </c>
+      <c r="M4" t="s" s="1">
+        <v>8</v>
+      </c>
+      <c r="N4" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="O4" t="s" s="1">
+        <v>21</v>
+      </c>
+      <c r="P4" t="s" s="1">
+        <v>22</v>
+      </c>
+      <c r="Q4" t="s" s="1">
+        <v>23</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>53</v>
+        <v>82</v>
       </c>
       <c r="B5" t="n" s="0">
         <v>0.0</v>
@@ -1389,22 +1407,31 @@
       <c r="C5" t="n" s="0">
         <v>1.0</v>
       </c>
-      <c r="D5" t="s" s="0">
-        <v>82</v>
-      </c>
       <c r="E5" t="s" s="0">
-        <v>54</v>
+        <v>83</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>54</v>
+        <v>84</v>
+      </c>
+      <c r="K5" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="L5" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="M5" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="N5" t="b" s="0">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B6" t="n" s="0">
         <v>0.0</v>
@@ -1412,19 +1439,52 @@
       <c r="C6" t="n" s="0">
         <v>1.0</v>
       </c>
-      <c r="D6" t="s" s="0">
-        <v>82</v>
-      </c>
       <c r="E6" t="s" s="0">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F6" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="K6" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="L6" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="M6" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="N6" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="B7" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="C7" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="F7" t="s" s="0">
         <v>55</v>
       </c>
-      <c r="H6" t="s" s="0">
-        <v>85</v>
-      </c>
-    </row>
+      <c r="H7" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="N7" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -1432,19 +1492,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="62.76953125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="31.78515625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="31.3515625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="16.46484375" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="20.98828125" customWidth="true" bestFit="true"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2">
@@ -1457,7 +1510,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>32</v>
@@ -1465,7 +1518,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>32</v>
@@ -1474,18 +1527,18 @@
     <row r="5"/>
     <row r="6">
       <c r="A6" t="s" s="1">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="1">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B7" t="s" s="1">
         <v>1</v>
       </c>
       <c r="C7" t="s" s="1">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D7" t="s" s="1">
         <v>2</v>
@@ -1493,13 +1546,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>32</v>
@@ -1507,13 +1560,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s" s="0">
         <v>32</v>
@@ -1522,12 +1575,12 @@
     <row r="10"/>
     <row r="11">
       <c r="A11" t="s" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="1">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13">
@@ -1537,33 +1590,36 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="1">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B14" t="s" s="1">
         <v>1</v>
       </c>
       <c r="C14" t="s" s="1">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D14" t="s" s="1">
         <v>54</v>
       </c>
       <c r="E14" t="s" s="1">
-        <v>84</v>
+        <v>83</v>
+      </c>
+      <c r="F14" t="s" s="1">
+        <v>86</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>9</v>
@@ -1571,16 +1627,16 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E16" t="s" s="0">
         <v>56</v>
@@ -1588,73 +1644,24 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="E17" t="s" s="0">
         <v>74</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>99</v>
-      </c>
-      <c r="C18" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>100</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>106</v>
-      </c>
-      <c r="B19" t="s" s="0">
-        <v>102</v>
-      </c>
-      <c r="C19" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>100</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s" s="0">
-        <v>107</v>
-      </c>
-      <c r="B20" t="s" s="0">
-        <v>104</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>100</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21"/>
+      <c r="F17" t="s">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -1672,7 +1679,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="1">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3">
@@ -1682,28 +1689,28 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s" s="1">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s" s="1">
         <v>1</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E4" t="s" s="1">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F4" t="s" s="1">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G4" t="s" s="1">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H4" t="s" s="1">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I4" t="s" s="1">
         <v>54</v>
@@ -1723,19 +1730,19 @@
     </row>
     <row r="5">
       <c r="B5" t="s" s="0">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="G5" t="s" s="0">
         <v>32</v>
@@ -1744,27 +1751,27 @@
         <v>32</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L5" t="s" s="0">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s" s="0">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="G6" t="s" s="0">
         <v>32</v>
@@ -1773,36 +1780,36 @@
         <v>32</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J6" t="s" s="0">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K6" t="s" s="0">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L6" t="s" s="0">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M6" t="s" s="0">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="s" s="0">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="G7" t="s" s="0">
         <v>32</v>
@@ -1811,13 +1818,13 @@
         <v>32</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K7" t="s" s="0">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8"/>
@@ -1828,7 +1835,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="1">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11">
@@ -1838,28 +1845,28 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="1">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B12" t="s" s="1">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C12" t="s" s="1">
         <v>1</v>
       </c>
       <c r="D12" t="s" s="1">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E12" t="s" s="1">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F12" t="s" s="1">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G12" t="s" s="1">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I12" t="s" s="1">
         <v>54</v>
@@ -1870,28 +1877,28 @@
     </row>
     <row r="13">
       <c r="B13" t="s" s="0">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F13" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H13" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="I13" t="s" s="0">
         <v>129</v>
-      </c>
-      <c r="G13" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="H13" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="I13" t="s" s="0">
-        <v>128</v>
       </c>
       <c r="J13" t="s" s="0">
         <v>130</v>
@@ -1905,13 +1912,13 @@
         <v>132</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="G14" t="s" s="0">
         <v>32</v>
@@ -1934,7 +1941,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="1">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18">
@@ -1944,28 +1951,28 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="1">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B19" t="s" s="1">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s" s="1">
         <v>1</v>
       </c>
       <c r="D19" t="s" s="1">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s" s="1">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F19" t="s" s="1">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G19" t="s" s="1">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H19" t="s" s="1">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I19" t="s" s="1">
         <v>54</v>
@@ -2000,137 +2007,137 @@
         <v>135</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F20" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="G20" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H20" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="I20" t="s" s="0">
         <v>136</v>
       </c>
-      <c r="G20" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="H20" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="I20" t="s" s="0">
+      <c r="J20" t="s" s="0">
+        <v>140</v>
+      </c>
+      <c r="K20" t="s">
         <v>137</v>
       </c>
-      <c r="J20" t="s" s="0">
+      <c r="L20" t="s">
+        <v>138</v>
+      </c>
+      <c r="M20" t="s">
+        <v>128</v>
+      </c>
+      <c r="N20" t="s">
+        <v>139</v>
+      </c>
+      <c r="O20" t="s">
         <v>141</v>
       </c>
-      <c r="K20" t="s">
-        <v>138</v>
-      </c>
-      <c r="L20" t="s">
-        <v>139</v>
-      </c>
-      <c r="M20" t="s">
-        <v>127</v>
-      </c>
-      <c r="N20" t="s">
-        <v>140</v>
-      </c>
-      <c r="O20" t="s">
-        <v>142</v>
-      </c>
       <c r="P20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="s" s="0">
+        <v>142</v>
+      </c>
+      <c r="C21" t="s" s="0">
         <v>143</v>
       </c>
-      <c r="C21" t="s" s="0">
+      <c r="D21" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H21" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="I21" t="s" s="0">
         <v>144</v>
       </c>
-      <c r="D21" t="s" s="0">
-        <v>87</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="F21" t="s" s="0">
-        <v>136</v>
-      </c>
-      <c r="G21" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="H21" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="I21" t="s" s="0">
+      <c r="J21" t="s" s="0">
         <v>145</v>
       </c>
-      <c r="J21" t="s" s="0">
-        <v>146</v>
-      </c>
       <c r="K21" t="s">
+        <v>137</v>
+      </c>
+      <c r="L21" t="s">
         <v>138</v>
-      </c>
-      <c r="L21" t="s">
-        <v>139</v>
       </c>
       <c r="M21" t="s">
         <v>131</v>
       </c>
       <c r="N21" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O21" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="C22" t="s" s="0">
         <v>148</v>
       </c>
-      <c r="C22" t="s" s="0">
+      <c r="D22" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="G22" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H22" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="I22" t="s" s="0">
         <v>149</v>
       </c>
-      <c r="D22" t="s" s="0">
-        <v>87</v>
-      </c>
-      <c r="E22" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="F22" t="s" s="0">
-        <v>136</v>
-      </c>
-      <c r="G22" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="H22" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="I22" t="s" s="0">
+      <c r="J22" t="s" s="0">
         <v>150</v>
       </c>
-      <c r="J22" t="s" s="0">
-        <v>151</v>
-      </c>
       <c r="K22" t="s">
+        <v>137</v>
+      </c>
+      <c r="L22" t="s">
         <v>138</v>
-      </c>
-      <c r="L22" t="s">
-        <v>139</v>
       </c>
       <c r="M22" t="s">
         <v>131</v>
       </c>
       <c r="N22" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O22" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
bis-2328: Persist RO-Crate ID in new property
</commit_message>
<xml_diff>
--- a/app-ro-crate-openbis/src/test/resources/json2excel/openbis_test_ro_out.xlsx
+++ b/app-ro-crate-openbis/src/test/resources/json2excel/openbis_test_ro_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="155">
   <si>
     <t>SAMPLE_TYPE</t>
   </si>
@@ -180,13 +180,22 @@
     <t>openBIS:hasPUBLICATION.CREATOR: PUBLICATION.CREATOR</t>
   </si>
   <si>
+    <t>RO-Crate.ID</t>
+  </si>
+  <si>
+    <t>RO-Crate ID</t>
+  </si>
+  <si>
+    <t>VARCHAR</t>
+  </si>
+  <si>
+    <t>RO-Crate ID: External identifier from RO-Crate</t>
+  </si>
+  <si>
     <t>NAME</t>
   </si>
   <si>
     <t>Name</t>
-  </si>
-  <si>
-    <t>VARCHAR</t>
   </si>
   <si>
     <t>PUBLICATION_CREATOR</t>
@@ -533,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -882,148 +891,148 @@
         <v>55</v>
       </c>
       <c r="H12" t="s" s="0">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="K12" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="L12" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="M12" t="s" s="0">
+        <v>32</v>
       </c>
       <c r="N12" t="b" s="0">
         <v>0</v>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" t="s" s="1">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="B13" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="C13" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="H13" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="N13" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="s" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="1">
         <v>1</v>
       </c>
-      <c r="B15" t="s" s="1">
+      <c r="B16" t="s" s="1">
         <v>2</v>
       </c>
-      <c r="C15" t="s" s="1">
+      <c r="C16" t="s" s="1">
         <v>3</v>
       </c>
-      <c r="D15" t="s" s="1">
+      <c r="D16" t="s" s="1">
         <v>4</v>
       </c>
-      <c r="E15" t="s" s="1">
+      <c r="E16" t="s" s="1">
         <v>5</v>
       </c>
-      <c r="F15" t="s" s="1">
+      <c r="F16" t="s" s="1">
         <v>6</v>
       </c>
-      <c r="G15" t="s" s="1">
+      <c r="G16" t="s" s="1">
         <v>7</v>
       </c>
-      <c r="H15" t="s" s="1">
+      <c r="H16" t="s" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>56</v>
-      </c>
-      <c r="B16" s="0"/>
-      <c r="C16" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="E16" t="b" s="0">
-        <v>0</v>
-      </c>
-      <c r="F16" t="s" s="0">
-        <v>57</v>
-      </c>
-      <c r="G16" t="s" s="0">
-        <v>58</v>
-      </c>
-      <c r="H16" t="s" s="0">
-        <v>58</v>
-      </c>
-    </row>
     <row r="17">
-      <c r="A17" t="s" s="1">
+      <c r="A17" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B17" s="0"/>
+      <c r="C17" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E17" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="G17" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="H17" t="s" s="0">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="1">
         <v>1</v>
       </c>
-      <c r="B17" t="s" s="1">
+      <c r="B18" t="s" s="1">
         <v>12</v>
       </c>
-      <c r="C17" t="s" s="1">
+      <c r="C18" t="s" s="1">
         <v>13</v>
       </c>
-      <c r="D17" t="s" s="1">
+      <c r="D18" t="s" s="1">
         <v>14</v>
       </c>
-      <c r="E17" t="s" s="1">
+      <c r="E18" t="s" s="1">
         <v>15</v>
       </c>
-      <c r="F17" t="s" s="1">
+      <c r="F18" t="s" s="1">
         <v>16</v>
       </c>
-      <c r="G17" t="s" s="1">
+      <c r="G18" t="s" s="1">
         <v>17</v>
       </c>
-      <c r="H17" t="s" s="1">
+      <c r="H18" t="s" s="1">
         <v>2</v>
       </c>
-      <c r="I17" t="s" s="1">
+      <c r="I18" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="J17" t="s" s="1">
+      <c r="J18" t="s" s="1">
         <v>19</v>
       </c>
-      <c r="K17" t="s" s="1">
+      <c r="K18" t="s" s="1">
         <v>6</v>
       </c>
-      <c r="L17" t="s" s="1">
+      <c r="L18" t="s" s="1">
         <v>7</v>
       </c>
-      <c r="M17" t="s" s="1">
+      <c r="M18" t="s" s="1">
         <v>8</v>
       </c>
-      <c r="N17" t="s" s="1">
+      <c r="N18" t="s" s="1">
         <v>20</v>
       </c>
-      <c r="O17" t="s" s="1">
+      <c r="O18" t="s" s="1">
         <v>21</v>
       </c>
-      <c r="P17" t="s" s="1">
+      <c r="P18" t="s" s="1">
         <v>22</v>
       </c>
-      <c r="Q17" t="s" s="1">
+      <c r="Q18" t="s" s="1">
         <v>23</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>59</v>
-      </c>
-      <c r="B18" t="n" s="0">
-        <v>0.0</v>
-      </c>
-      <c r="C18" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="F18" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="H18" t="s" s="0">
-        <v>61</v>
-      </c>
-      <c r="K18" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="L18" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="M18" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="N18" t="b" s="0">
-        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1046,13 +1055,13 @@
         <v>64</v>
       </c>
       <c r="K19" t="s" s="0">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="L19" t="s" s="0">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="M19" t="s" s="0">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="N19" t="b" s="0">
         <v>0</v>
@@ -1060,7 +1069,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B20" t="n" s="0">
         <v>0.0</v>
@@ -1069,22 +1078,22 @@
         <v>1.0</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F20" t="s" s="0">
         <v>26</v>
       </c>
       <c r="H20" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="K20" t="s" s="0">
         <v>68</v>
       </c>
-      <c r="K20" t="s" s="0">
-        <v>69</v>
-      </c>
       <c r="L20" t="s" s="0">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M20" t="s" s="0">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="N20" t="b" s="0">
         <v>0</v>
@@ -1092,7 +1101,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B21" t="n" s="0">
         <v>0.0</v>
@@ -1101,22 +1110,22 @@
         <v>1.0</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F21" t="s" s="0">
         <v>26</v>
       </c>
       <c r="H21" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="K21" t="s" s="0">
         <v>72</v>
       </c>
-      <c r="K21" t="s" s="0">
-        <v>73</v>
-      </c>
       <c r="L21" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M21" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N21" t="b" s="0">
         <v>0</v>
@@ -1124,7 +1133,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="B22" t="n" s="0">
         <v>0.0</v>
@@ -1133,69 +1142,86 @@
         <v>1.0</v>
       </c>
       <c r="E22" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="H22" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="K22" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="L22" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="M22" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="N22" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="B23" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="C23" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E23" t="s" s="0">
         <v>54</v>
       </c>
-      <c r="F22" t="s" s="0">
+      <c r="F23" t="s" s="0">
         <v>55</v>
       </c>
-      <c r="H22" t="s" s="0">
-        <v>54</v>
-      </c>
-      <c r="N22" t="b" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23"/>
+      <c r="H23" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="K23" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="L23" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="M23" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="N23" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" t="s" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s" s="1">
-        <v>1</v>
-      </c>
-      <c r="B25" t="s" s="1">
-        <v>2</v>
-      </c>
-      <c r="C25" t="s" s="1">
-        <v>3</v>
-      </c>
-      <c r="D25" t="s" s="1">
-        <v>4</v>
-      </c>
-      <c r="E25" t="s" s="1">
-        <v>5</v>
-      </c>
-      <c r="F25" t="s" s="1">
-        <v>6</v>
-      </c>
-      <c r="G25" t="s" s="1">
-        <v>7</v>
-      </c>
-      <c r="H25" t="s" s="1">
-        <v>8</v>
-      </c>
-    </row>
+      <c r="A24" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="B24" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="C24" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="F24" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="H24" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="N24" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25"/>
     <row r="26">
-      <c r="A26" t="s" s="0">
-        <v>74</v>
-      </c>
-      <c r="B26" s="0"/>
-      <c r="C26" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="E26" t="b" s="0">
-        <v>0</v>
-      </c>
-      <c r="F26" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="G26" t="s" s="0">
-        <v>75</v>
-      </c>
-      <c r="H26" t="s" s="0">
-        <v>75</v>
+      <c r="A26" t="s" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1203,110 +1229,189 @@
         <v>1</v>
       </c>
       <c r="B27" t="s" s="1">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C27" t="s" s="1">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="D27" t="s" s="1">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E27" t="s" s="1">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F27" t="s" s="1">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G27" t="s" s="1">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="H27" t="s" s="1">
-        <v>2</v>
-      </c>
-      <c r="I27" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="J27" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="K27" t="s" s="1">
-        <v>6</v>
-      </c>
-      <c r="L27" t="s" s="1">
-        <v>7</v>
-      </c>
-      <c r="M27" t="s" s="1">
         <v>8</v>
-      </c>
-      <c r="N27" t="s" s="1">
-        <v>20</v>
-      </c>
-      <c r="O27" t="s" s="1">
-        <v>21</v>
-      </c>
-      <c r="P27" t="s" s="1">
-        <v>22</v>
-      </c>
-      <c r="Q27" t="s" s="1">
-        <v>23</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>76</v>
-      </c>
-      <c r="B28" t="n" s="0">
-        <v>0.0</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="B28" s="0"/>
       <c r="C28" t="n" s="0">
         <v>1.0</v>
       </c>
-      <c r="E28" t="s" s="0">
-        <v>77</v>
+      <c r="E28" t="b" s="0">
+        <v>0</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>26</v>
+        <v>10</v>
+      </c>
+      <c r="G28" t="s" s="0">
+        <v>78</v>
       </c>
       <c r="H28" t="s" s="0">
         <v>78</v>
       </c>
-      <c r="K28" t="s" s="0">
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="1">
+        <v>1</v>
+      </c>
+      <c r="B29" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="C29" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="D29" t="s" s="1">
+        <v>14</v>
+      </c>
+      <c r="E29" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="F29" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="G29" t="s" s="1">
+        <v>17</v>
+      </c>
+      <c r="H29" t="s" s="1">
+        <v>2</v>
+      </c>
+      <c r="I29" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="J29" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="K29" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="L29" t="s" s="1">
+        <v>7</v>
+      </c>
+      <c r="M29" t="s" s="1">
+        <v>8</v>
+      </c>
+      <c r="N29" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="O29" t="s" s="1">
+        <v>21</v>
+      </c>
+      <c r="P29" t="s" s="1">
+        <v>22</v>
+      </c>
+      <c r="Q29" t="s" s="1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
         <v>79</v>
       </c>
-      <c r="L28" t="s" s="0">
-        <v>79</v>
-      </c>
-      <c r="M28" t="s" s="0">
-        <v>79</v>
-      </c>
-      <c r="N28" t="b" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s" s="0">
+      <c r="B30" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="C30" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E30" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="F30" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="H30" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="K30" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="L30" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="M30" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="N30" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
         <v>53</v>
       </c>
-      <c r="B29" t="n" s="0">
+      <c r="B31" t="n" s="0">
         <v>0.0</v>
       </c>
-      <c r="C29" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="E29" t="s" s="0">
+      <c r="C31" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E31" t="s" s="0">
         <v>54</v>
       </c>
-      <c r="F29" t="s" s="0">
+      <c r="F31" t="s" s="0">
         <v>55</v>
       </c>
-      <c r="H29" t="s" s="0">
-        <v>54</v>
-      </c>
-      <c r="N29" t="b" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30"/>
+      <c r="H31" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="K31" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="L31" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="M31" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="N31" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="B32" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="C32" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="F32" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="H32" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="N32" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -1314,12 +1419,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2">
@@ -1335,7 +1440,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>32</v>
@@ -1399,7 +1504,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B5" t="n" s="0">
         <v>0.0</v>
@@ -1408,13 +1513,13 @@
         <v>1.0</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>26</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="K5" t="s" s="0">
         <v>32</v>
@@ -1431,7 +1536,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B6" t="n" s="0">
         <v>0.0</v>
@@ -1440,13 +1545,13 @@
         <v>1.0</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F6" t="s" s="0">
         <v>26</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K6" t="s" s="0">
         <v>32</v>
@@ -1478,13 +1583,45 @@
         <v>55</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="K7" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="L7" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="M7" t="s" s="0">
+        <v>32</v>
       </c>
       <c r="N7" t="b" s="0">
         <v>0</v>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="B8" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="C8" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="N8" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -1492,12 +1629,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2">
@@ -1510,7 +1647,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>32</v>
@@ -1518,7 +1655,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>32</v>
@@ -1527,18 +1664,18 @@
     <row r="5"/>
     <row r="6">
       <c r="A6" t="s" s="1">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="1">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s" s="1">
         <v>1</v>
       </c>
       <c r="C7" t="s" s="1">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D7" t="s" s="1">
         <v>2</v>
@@ -1546,13 +1683,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>32</v>
@@ -1560,13 +1697,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D9" t="s" s="0">
         <v>32</v>
@@ -1575,90 +1712,102 @@
     <row r="10"/>
     <row r="11">
       <c r="A11" t="s" s="1">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="1">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="1">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B14" t="s" s="1">
         <v>1</v>
       </c>
       <c r="C14" t="s" s="1">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D14" t="s" s="1">
+        <v>58</v>
+      </c>
+      <c r="E14" t="s" s="1">
+        <v>86</v>
+      </c>
+      <c r="F14" t="s" s="1">
+        <v>89</v>
+      </c>
+      <c r="G14" t="s" s="1">
         <v>54</v>
-      </c>
-      <c r="E14" t="s" s="1">
-        <v>83</v>
-      </c>
-      <c r="F14" t="s" s="1">
-        <v>86</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>9</v>
       </c>
+      <c r="G15" t="s" s="0">
+        <v>103</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>56</v>
+        <v>59</v>
+      </c>
+      <c r="G16" t="s" s="0">
+        <v>106</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F17" t="s">
+        <v>112</v>
+      </c>
+      <c r="G17" t="s">
         <v>109</v>
       </c>
     </row>
@@ -1669,7 +1818,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1679,70 +1828,73 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="1">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B4" t="s" s="1">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C4" t="s" s="1">
         <v>1</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E4" t="s" s="1">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F4" t="s" s="1">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="G4" t="s" s="1">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="H4" t="s" s="1">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I4" t="s" s="1">
+        <v>58</v>
+      </c>
+      <c r="J4" t="s" s="1">
+        <v>63</v>
+      </c>
+      <c r="K4" t="s" s="1">
+        <v>66</v>
+      </c>
+      <c r="L4" t="s" s="1">
+        <v>70</v>
+      </c>
+      <c r="M4" t="s" s="1">
+        <v>74</v>
+      </c>
+      <c r="N4" t="s" s="1">
         <v>54</v>
-      </c>
-      <c r="J4" t="s" s="1">
-        <v>60</v>
-      </c>
-      <c r="K4" t="s" s="1">
-        <v>63</v>
-      </c>
-      <c r="L4" t="s" s="1">
-        <v>67</v>
-      </c>
-      <c r="M4" t="s" s="1">
-        <v>71</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="s" s="0">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G5" t="s" s="0">
         <v>32</v>
@@ -1751,27 +1903,30 @@
         <v>32</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="L5" t="s" s="0">
-        <v>117</v>
+        <v>120</v>
+      </c>
+      <c r="N5" t="s" s="0">
+        <v>118</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s" s="0">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G6" t="s" s="0">
         <v>32</v>
@@ -1780,36 +1935,39 @@
         <v>32</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="J6" t="s" s="0">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="K6" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="L6" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="M6" t="s" s="0">
+        <v>126</v>
+      </c>
+      <c r="N6" t="s" s="0">
         <v>121</v>
-      </c>
-      <c r="L6" t="s" s="0">
-        <v>122</v>
-      </c>
-      <c r="M6" t="s" s="0">
-        <v>123</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="s" s="0">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G7" t="s" s="0">
         <v>32</v>
@@ -1818,12 +1976,15 @@
         <v>32</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="K7" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="N7" t="s" s="0">
         <v>127</v>
       </c>
     </row>
@@ -1835,61 +1996,64 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="1">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="1">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B12" t="s" s="1">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s" s="1">
         <v>1</v>
       </c>
       <c r="D12" t="s" s="1">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E12" t="s" s="1">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F12" t="s" s="1">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="G12" t="s" s="1">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I12" t="s" s="1">
+        <v>58</v>
+      </c>
+      <c r="J12" t="s" s="1">
+        <v>80</v>
+      </c>
+      <c r="K12" t="s" s="1">
         <v>54</v>
-      </c>
-      <c r="J12" t="s" s="1">
-        <v>77</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="s" s="0">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G13" t="s" s="0">
         <v>32</v>
@@ -1898,27 +2062,30 @@
         <v>32</v>
       </c>
       <c r="I13" t="s" s="0">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J13" t="s" s="0">
-        <v>130</v>
+        <v>133</v>
+      </c>
+      <c r="K13" t="s" s="0">
+        <v>131</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="s" s="0">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G14" t="s" s="0">
         <v>32</v>
@@ -1927,10 +2094,13 @@
         <v>32</v>
       </c>
       <c r="I14" t="s" s="0">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="J14" t="s" s="0">
-        <v>133</v>
+        <v>136</v>
+      </c>
+      <c r="K14" t="s" s="0">
+        <v>134</v>
       </c>
     </row>
     <row r="15"/>
@@ -1941,7 +2111,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="1">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18">
@@ -1951,31 +2121,31 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="1">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B19" t="s" s="1">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C19" t="s" s="1">
         <v>1</v>
       </c>
       <c r="D19" t="s" s="1">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E19" t="s" s="1">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F19" t="s" s="1">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="G19" t="s" s="1">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="H19" t="s" s="1">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I19" t="s" s="1">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="J19" t="s" s="1">
         <v>25</v>
@@ -1998,22 +2168,25 @@
       <c r="P19" t="s" s="1">
         <v>51</v>
       </c>
+      <c r="Q19" t="s" s="1">
+        <v>54</v>
+      </c>
     </row>
     <row r="20">
       <c r="B20" t="s" s="0">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G20" t="s" s="0">
         <v>32</v>
@@ -2022,92 +2195,98 @@
         <v>32</v>
       </c>
       <c r="I20" t="s" s="0">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="J20" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="K20" t="s">
         <v>140</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
+        <v>141</v>
+      </c>
+      <c r="M20" t="s">
+        <v>131</v>
+      </c>
+      <c r="N20" t="s">
+        <v>142</v>
+      </c>
+      <c r="O20" t="s">
+        <v>144</v>
+      </c>
+      <c r="P20" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q20" t="s">
         <v>137</v>
-      </c>
-      <c r="L20" t="s">
-        <v>138</v>
-      </c>
-      <c r="M20" t="s">
-        <v>128</v>
-      </c>
-      <c r="N20" t="s">
-        <v>139</v>
-      </c>
-      <c r="O20" t="s">
-        <v>141</v>
-      </c>
-      <c r="P20" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="s" s="0">
+        <v>145</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>146</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>103</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H21" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="I21" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="J21" t="s" s="0">
+        <v>148</v>
+      </c>
+      <c r="K21" t="s">
+        <v>140</v>
+      </c>
+      <c r="L21" t="s">
+        <v>141</v>
+      </c>
+      <c r="M21" t="s">
+        <v>134</v>
+      </c>
+      <c r="N21" t="s">
         <v>142</v>
       </c>
-      <c r="C21" t="s" s="0">
-        <v>143</v>
-      </c>
-      <c r="D21" t="s" s="0">
-        <v>89</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="F21" t="s" s="0">
-        <v>100</v>
-      </c>
-      <c r="G21" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="H21" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="I21" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="J21" t="s" s="0">
+      <c r="O21" t="s">
+        <v>149</v>
+      </c>
+      <c r="P21" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q21" t="s">
         <v>145</v>
-      </c>
-      <c r="K21" t="s">
-        <v>137</v>
-      </c>
-      <c r="L21" t="s">
-        <v>138</v>
-      </c>
-      <c r="M21" t="s">
-        <v>131</v>
-      </c>
-      <c r="N21" t="s">
-        <v>139</v>
-      </c>
-      <c r="O21" t="s">
-        <v>146</v>
-      </c>
-      <c r="P21" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="s" s="0">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G22" t="s" s="0">
         <v>32</v>
@@ -2116,28 +2295,31 @@
         <v>32</v>
       </c>
       <c r="I22" t="s" s="0">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J22" t="s" s="0">
+        <v>153</v>
+      </c>
+      <c r="K22" t="s">
+        <v>140</v>
+      </c>
+      <c r="L22" t="s">
+        <v>141</v>
+      </c>
+      <c r="M22" t="s">
+        <v>134</v>
+      </c>
+      <c r="N22" t="s">
+        <v>142</v>
+      </c>
+      <c r="O22" t="s">
+        <v>154</v>
+      </c>
+      <c r="P22" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q22" t="s">
         <v>150</v>
-      </c>
-      <c r="K22" t="s">
-        <v>137</v>
-      </c>
-      <c r="L22" t="s">
-        <v>138</v>
-      </c>
-      <c r="M22" t="s">
-        <v>131</v>
-      </c>
-      <c r="N22" t="s">
-        <v>139</v>
-      </c>
-      <c r="O22" t="s">
-        <v>151</v>
-      </c>
-      <c r="P22" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>